<commit_message>
FULL RESTORE: recover 291 files lost in external reset (post covers/audio/body, blog/_tools, functions/api, _redirects, 16-Jul fixed pages) from orphaned 1c9862c; keep newer tracker/data from current lineage
</commit_message>
<xml_diff>
--- a/tools/fii-flows/FII_FPI_Historical_Data_India.xlsx
+++ b/tools/fii-flows/FII_FPI_Historical_Data_India.xlsx
@@ -1098,16 +1098,16 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>-93810</v>
+        <v>-143150</v>
       </c>
       <c r="C36" t="n">
-        <v>-6559</v>
+        <v>47450</v>
       </c>
       <c r="D36" t="n">
-        <v>-100369</v>
+        <v>-95700</v>
       </c>
       <c r="E36" t="n">
-        <v>1384034</v>
+        <v>1388703</v>
       </c>
     </row>
   </sheetData>
@@ -1564,16 +1564,16 @@
         <v>2026</v>
       </c>
       <c r="B26" t="n">
-        <v>-224932</v>
+        <v>-274272</v>
       </c>
       <c r="C26" t="n">
-        <v>7391</v>
+        <v>61400</v>
       </c>
       <c r="D26" t="n">
-        <v>-217541</v>
+        <v>-212872</v>
       </c>
       <c r="E26" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1587,7 +1587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C294"/>
+  <dimension ref="A1:C295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5416,6 +5416,19 @@
         <v>-29484</v>
       </c>
     </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>-49340</v>
+      </c>
+      <c r="C295" t="n">
+        <v>4669</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>